<commit_message>
fix: finished week 8 deliverables
</commit_message>
<xml_diff>
--- a/Documentation/Week 8/Booked Hours/Booked_Hours_Dylan.xlsx
+++ b/Documentation/Week 8/Booked Hours/Booked_Hours_Dylan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24314441_student_uwa_edu_au/Documents/UWA/Year 3/Sem 2/CITS3200_Project/Documentation/Week 8/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24B8FE87-EA41-45BE-B418-A6543B382B64}"/>
+  <xr:revisionPtr revIDLastSave="306" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8774C72E-7810-462D-9B97-A665F7B585B5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="29">
   <si>
     <r>
       <t xml:space="preserve">CITS3200 Project Billed Hours Record for &lt;Dylan Hu&gt;
@@ -131,13 +131,13 @@
     <t>Project testing and debugging</t>
   </si>
   <si>
-    <t>Client meeting Prep (documentation)</t>
-  </si>
-  <si>
     <t>Team and client meeting prep</t>
   </si>
   <si>
     <t>Submitting weekly deliverables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client meeting </t>
   </si>
 </sst>
 </file>
@@ -378,6 +378,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -396,14 +404,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -841,36 +841,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="13"/>
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="16" t="s">
+      <c r="C2" s="12"/>
+      <c r="D2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="17"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="18" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="16" t="s">
         <v>6</v>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="F3" s="19"/>
       <c r="G3" s="10"/>
-      <c r="H3" s="15"/>
+      <c r="H3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1716,7 +1716,7 @@
         <v>0.75</v>
       </c>
       <c r="H29" s="1">
-        <f t="shared" ref="H29:I30" si="8">IF(AND(G29&lt;&gt;" ",G29&lt;&gt;"ERROR",H28&lt;&gt;" ", H28&lt;&gt;"ERROR"),G29+H28," ")</f>
+        <f t="shared" ref="H29:H30" si="8">IF(AND(G29&lt;&gt;" ",G29&lt;&gt;"ERROR",H28&lt;&gt;" ", H28&lt;&gt;"ERROR"),G29+H28," ")</f>
         <v>26.249999999825377</v>
       </c>
       <c r="I29" s="1">
@@ -1741,7 +1741,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G30" s="6">
         <f t="shared" si="0"/>
@@ -1760,14 +1760,14 @@
       <c r="A31" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="16" t="s">
+      <c r="C31" s="12"/>
+      <c r="D31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="17"/>
+      <c r="E31" s="12"/>
       <c r="F31" s="8" t="s">
         <v>4</v>
       </c>
@@ -1853,14 +1853,14 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G34" s="6">
         <f t="shared" si="9"/>
         <v>1.0000000001164153</v>
       </c>
       <c r="H34" s="1">
-        <f t="shared" ref="H33:H35" si="10">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
+        <f t="shared" ref="H34:H35" si="10">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
         <v>28.5</v>
       </c>
       <c r="I34" s="1">
@@ -1885,7 +1885,7 @@
         <v>0.98958333333333337</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G35" s="6">
         <f t="shared" si="9"/>
@@ -1906,11 +1906,11 @@
       <c r="D36" s="4"/>
       <c r="E36" s="5"/>
       <c r="G36" s="6" t="str">
-        <f t="shared" ref="G33:G64" si="11">IF(I36&gt;0,I36,IF(I36=0, " ", "ERROR"))</f>
+        <f t="shared" ref="G36:G64" si="11">IF(I36&gt;0,I36,IF(I36=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H36" s="1" t="str">
-        <f t="shared" ref="H34:H64" si="12">IF(AND(G36&lt;&gt;" ",G36&lt;&gt;"ERROR",H35&lt;&gt;" ", H35&lt;&gt;"ERROR"),G36+H35," ")</f>
+        <f t="shared" ref="H36:H64" si="12">IF(AND(G36&lt;&gt;" ",G36&lt;&gt;"ERROR",H35&lt;&gt;" ", H35&lt;&gt;"ERROR"),G36+H35," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I36" s="1">
@@ -2411,14 +2411,14 @@
       <c r="A65" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C65" s="17"/>
-      <c r="D65" s="16" t="s">
+      <c r="C65" s="12"/>
+      <c r="D65" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E65" s="17"/>
+      <c r="E65" s="12"/>
       <c r="F65" s="8" t="s">
         <v>4</v>
       </c>
@@ -2907,14 +2907,14 @@
       <c r="A99" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B99" s="16" t="s">
+      <c r="B99" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C99" s="17"/>
-      <c r="D99" s="16" t="s">
+      <c r="C99" s="12"/>
+      <c r="D99" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E99" s="17"/>
+      <c r="E99" s="12"/>
       <c r="F99" s="8" t="s">
         <v>4</v>
       </c>
@@ -3401,18 +3401,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -3426,6 +3414,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>